<commit_message>
phase 2 input files
</commit_message>
<xml_diff>
--- a/phase1/job simulation.xlsx
+++ b/phase1/job simulation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alesh\OneDrive\Documents\coding\college\os\phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E398B1-3940-44BD-98CD-A71DE7985EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55630E7-B4E6-4289-B746-A7F6DBB74E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{42410815-3CF0-40EE-AB44-C05703D69E0B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="59">
   <si>
     <t>R</t>
   </si>
@@ -78,15 +78,6 @@
     <t>H</t>
   </si>
   <si>
-    <t>e</t>
-  </si>
-  <si>
-    <t>r</t>
-  </si>
-  <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>VIT</t>
   </si>
   <si>
@@ -108,9 +99,6 @@
     <t>L</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>$AMJ000200110001</t>
   </si>
   <si>
@@ -120,18 +108,6 @@
     <t>program 2 - Same String</t>
   </si>
   <si>
-    <t>h</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>s</t>
-  </si>
-  <si>
-    <t>p</t>
-  </si>
-  <si>
     <t>car</t>
   </si>
   <si>
@@ -168,9 +144,6 @@
     <t>program 4 - String Replace</t>
   </si>
   <si>
-    <t>GDXXGDXXGDXXLRXXCRXXBTXXLRXXSRXXCRXXBTXXLRXXSRXXCRXXBTXXLRXXSRXXPDXXH</t>
-  </si>
-  <si>
     <t>GD20GD30GD40GD50LR20CR30BT09PD50HPD40</t>
   </si>
   <si>
@@ -189,15 +162,6 @@
     <t>$AMJ000400280001</t>
   </si>
   <si>
-    <t>l</t>
-  </si>
-  <si>
-    <t>i</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
     <t>GD30GD40LR30CR40BT11CR41BT15CR42BT19CR43</t>
   </si>
   <si>
@@ -214,6 +178,39 @@
   </si>
   <si>
     <t>$END0005</t>
+  </si>
+  <si>
+    <t>program 6 - Star Pattern</t>
+  </si>
+  <si>
+    <t>program 7 - Print Sentence In Reverse</t>
+  </si>
+  <si>
+    <t>$END0006</t>
+  </si>
+  <si>
+    <t>$END0007</t>
+  </si>
+  <si>
+    <t>HOW ARE YOU NOW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H </t>
+  </si>
+  <si>
+    <t>GD20LR20SR33LR21SR32LR22SR31LR23SR30PD30</t>
+  </si>
+  <si>
+    <t>$AMJ000700110001</t>
+  </si>
+  <si>
+    <t>$AMJ000600160006</t>
+  </si>
+  <si>
+    <t>GD20LR20SR30SR31SR40SR41SR42PD20PD30PD40</t>
+  </si>
+  <si>
+    <t>PD30PD20PD20PD20PD20H</t>
   </si>
 </sst>
 </file>
@@ -651,13 +648,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C25E82-8B1E-4B3C-94D6-569AB7836210}">
-  <dimension ref="A1:R101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
@@ -676,33 +673,30 @@
         <v>11</v>
       </c>
       <c r="O2" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P2" s="6">
         <v>0</v>
       </c>
-      <c r="R2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O3" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P3" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -717,7 +711,7 @@
         <v>2</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>0</v>
@@ -726,10 +720,10 @@
         <v>3</v>
       </c>
       <c r="P4" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -737,19 +731,19 @@
         <v>3</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O5" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P5" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -762,19 +756,19 @@
         <v>4</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O6" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P6" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -782,19 +776,19 @@
         <v>5</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O7" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -806,36 +800,36 @@
         <v>6</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O8" s="6">
+        <v>3</v>
+      </c>
+      <c r="P8" s="6">
         <v>1</v>
       </c>
-      <c r="P8" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="L9">
         <v>7</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O9" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F10" t="s">
         <v>4</v>
       </c>
@@ -844,267 +838,183 @@
         <v>8</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O10" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" s="6">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L11">
         <v>9</v>
       </c>
       <c r="M11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="O11" s="6">
         <v>3</v>
       </c>
-      <c r="N11" s="6" t="s">
+      <c r="P11" s="6">
         <v>0</v>
       </c>
-      <c r="O11" s="6">
-        <v>4</v>
-      </c>
-      <c r="P11" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L12">
         <v>10</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N12" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="O12" s="5">
-        <v>2</v>
-      </c>
-      <c r="P12" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="L13">
         <v>11</v>
       </c>
-      <c r="M13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="O13" s="5">
-        <v>5</v>
-      </c>
-      <c r="P13" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="L14">
         <v>12</v>
       </c>
-      <c r="M14" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="N14" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5">
-        <v>4</v>
-      </c>
-      <c r="P14" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
       <c r="L15">
         <v>13</v>
       </c>
-      <c r="M15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="O15" s="5">
-        <v>4</v>
-      </c>
-      <c r="P15" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>7</v>
       </c>
       <c r="L16">
         <v>14</v>
       </c>
-      <c r="M16" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="5"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L17">
         <v>15</v>
       </c>
-      <c r="M17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="N17" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="O17" s="5">
-        <v>5</v>
-      </c>
-      <c r="P17" s="5">
-        <v>0</v>
-      </c>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="L18">
         <v>16</v>
       </c>
-      <c r="M18" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="N18" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="O18" s="5">
-        <v>4</v>
-      </c>
-      <c r="P18" s="5">
-        <v>1</v>
-      </c>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L19">
         <v>17</v>
       </c>
-      <c r="M19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="O19" s="5">
-        <v>4</v>
-      </c>
-      <c r="P19" s="5">
-        <v>0</v>
-      </c>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L20">
         <v>18</v>
       </c>
-      <c r="M20" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="M20" s="5"/>
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
       <c r="P20" s="5"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L21">
         <v>19</v>
       </c>
-      <c r="M21" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="N21" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="O21" s="5">
-        <v>5</v>
-      </c>
-      <c r="P21" s="5">
-        <v>0</v>
-      </c>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L22">
         <v>20</v>
       </c>
-      <c r="M22" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N22" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="O22" s="6">
-        <v>4</v>
-      </c>
-      <c r="P22" s="6">
-        <v>2</v>
-      </c>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L23">
         <v>21</v>
       </c>
-      <c r="M23" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N23" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="O23" s="6">
-        <v>4</v>
-      </c>
-      <c r="P23" s="6">
-        <v>0</v>
-      </c>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="L24">
         <v>22</v>
       </c>
-      <c r="M24" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="M24" s="6"/>
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
       <c r="P24" s="6"/>
@@ -1113,69 +1023,43 @@
       <c r="L25">
         <v>23</v>
       </c>
-      <c r="M25" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N25" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="O25" s="6">
-        <v>5</v>
-      </c>
-      <c r="P25" s="6">
-        <v>0</v>
-      </c>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="L26">
         <v>24</v>
       </c>
-      <c r="M26" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N26" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="O26" s="6">
-        <v>4</v>
-      </c>
-      <c r="P26" s="6">
-        <v>3</v>
-      </c>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="L27">
         <v>25</v>
       </c>
-      <c r="M27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N27" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="O27" s="6">
-        <v>4</v>
-      </c>
-      <c r="P27" s="6">
-        <v>0</v>
-      </c>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="L28">
         <v>26</v>
       </c>
-      <c r="M28" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="M28" s="6"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
@@ -1194,7 +1078,7 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="L30">
         <v>28</v>
@@ -1206,7 +1090,7 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="L31">
         <v>29</v>
@@ -1220,15 +1104,9 @@
       <c r="L32">
         <v>30</v>
       </c>
-      <c r="M32" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="N32" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="O32" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
       <c r="P32" s="5"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.35">
@@ -1242,7 +1120,7 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="L34">
         <v>32</v>
@@ -1263,7 +1141,7 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="L36">
         <v>34</v>
@@ -1275,7 +1153,7 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="L37">
         <v>35</v>
@@ -1287,7 +1165,7 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="L38">
         <v>36</v>
@@ -1299,7 +1177,7 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="L39">
         <v>37</v>
@@ -1323,7 +1201,7 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="L41">
         <v>39</v>
@@ -1335,74 +1213,48 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="L42">
         <v>40</v>
       </c>
-      <c r="M42" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N42" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O42" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
       <c r="P42" s="6"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="L43">
         <v>41</v>
       </c>
-      <c r="M43" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N43" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="O43" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="P43" s="6" t="s">
-        <v>51</v>
-      </c>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="L44">
         <v>42</v>
       </c>
-      <c r="M44" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="M44" s="6"/>
       <c r="N44" s="6"/>
-      <c r="O44" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="P44" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L45">
         <v>43</v>
       </c>
       <c r="M45" s="6"/>
-      <c r="N45" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="O45" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="P45" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="N45" s="6"/>
+      <c r="O45" s="6"/>
+      <c r="P45" s="6"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L46">
@@ -1415,7 +1267,7 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="L47">
         <v>45</v>
@@ -1436,7 +1288,7 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="L49">
         <v>47</v>
@@ -1448,7 +1300,7 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="L50">
         <v>48</v>
@@ -1460,7 +1312,7 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="L51">
         <v>49</v>
@@ -1472,7 +1324,7 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="L52">
         <v>50</v>
@@ -1496,7 +1348,7 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="L54">
         <v>52</v>
@@ -1508,7 +1360,7 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L55">
         <v>53</v>
@@ -1520,7 +1372,7 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="L56">
         <v>54</v>
@@ -1549,6 +1401,9 @@
       <c r="P58" s="5"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>48</v>
+      </c>
       <c r="L59">
         <v>57</v>
       </c>
@@ -1567,6 +1422,9 @@
       <c r="P60" s="5"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>56</v>
+      </c>
       <c r="L61">
         <v>59</v>
       </c>
@@ -1576,6 +1434,9 @@
       <c r="P61" s="5"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>57</v>
+      </c>
       <c r="L62">
         <v>60</v>
       </c>
@@ -1585,6 +1446,9 @@
       <c r="P62" s="6"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>58</v>
+      </c>
       <c r="L63">
         <v>61</v>
       </c>
@@ -1594,6 +1458,9 @@
       <c r="P63" s="6"/>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>7</v>
+      </c>
       <c r="L64">
         <v>62</v>
       </c>
@@ -1602,7 +1469,10 @@
       <c r="O64" s="6"/>
       <c r="P64" s="6"/>
     </row>
-    <row r="65" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>30</v>
+      </c>
       <c r="L65">
         <v>63</v>
       </c>
@@ -1611,7 +1481,10 @@
       <c r="O65" s="6"/>
       <c r="P65" s="6"/>
     </row>
-    <row r="66" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>50</v>
+      </c>
       <c r="L66">
         <v>64</v>
       </c>
@@ -1620,7 +1493,7 @@
       <c r="O66" s="6"/>
       <c r="P66" s="6"/>
     </row>
-    <row r="67" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L67">
         <v>65</v>
       </c>
@@ -1629,7 +1502,7 @@
       <c r="O67" s="6"/>
       <c r="P67" s="6"/>
     </row>
-    <row r="68" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L68">
         <v>66</v>
       </c>
@@ -1638,7 +1511,10 @@
       <c r="O68" s="6"/>
       <c r="P68" s="6"/>
     </row>
-    <row r="69" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>49</v>
+      </c>
       <c r="L69">
         <v>67</v>
       </c>
@@ -1647,7 +1523,7 @@
       <c r="O69" s="6"/>
       <c r="P69" s="6"/>
     </row>
-    <row r="70" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L70">
         <v>68</v>
       </c>
@@ -1656,7 +1532,10 @@
       <c r="O70" s="6"/>
       <c r="P70" s="6"/>
     </row>
-    <row r="71" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>55</v>
+      </c>
       <c r="L71">
         <v>69</v>
       </c>
@@ -1665,7 +1544,10 @@
       <c r="O71" s="6"/>
       <c r="P71" s="6"/>
     </row>
-    <row r="72" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>54</v>
+      </c>
       <c r="L72">
         <v>70</v>
       </c>
@@ -1674,7 +1556,10 @@
       <c r="O72" s="5"/>
       <c r="P72" s="5"/>
     </row>
-    <row r="73" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>53</v>
+      </c>
       <c r="L73">
         <v>71</v>
       </c>
@@ -1683,7 +1568,10 @@
       <c r="O73" s="5"/>
       <c r="P73" s="5"/>
     </row>
-    <row r="74" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>7</v>
+      </c>
       <c r="L74">
         <v>72</v>
       </c>
@@ -1692,7 +1580,10 @@
       <c r="O74" s="5"/>
       <c r="P74" s="5"/>
     </row>
-    <row r="75" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>52</v>
+      </c>
       <c r="L75">
         <v>73</v>
       </c>
@@ -1701,7 +1592,10 @@
       <c r="O75" s="5"/>
       <c r="P75" s="5"/>
     </row>
-    <row r="76" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>51</v>
+      </c>
       <c r="L76">
         <v>74</v>
       </c>
@@ -1710,7 +1604,7 @@
       <c r="O76" s="5"/>
       <c r="P76" s="5"/>
     </row>
-    <row r="77" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L77">
         <v>75</v>
       </c>
@@ -1719,7 +1613,7 @@
       <c r="O77" s="5"/>
       <c r="P77" s="5"/>
     </row>
-    <row r="78" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L78">
         <v>76</v>
       </c>
@@ -1728,7 +1622,7 @@
       <c r="O78" s="5"/>
       <c r="P78" s="5"/>
     </row>
-    <row r="79" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L79">
         <v>77</v>
       </c>
@@ -1737,7 +1631,7 @@
       <c r="O79" s="5"/>
       <c r="P79" s="5"/>
     </row>
-    <row r="80" spans="12:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L80">
         <v>78</v>
       </c>
@@ -1937,5 +1831,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
phase 2 complete fr
</commit_message>
<xml_diff>
--- a/phase1/job simulation.xlsx
+++ b/phase1/job simulation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alesh\OneDrive\Documents\coding\college\os\phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55630E7-B4E6-4289-B746-A7F6DBB74E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A67C857-CC40-43C8-BE7E-8CC2CB760B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{42410815-3CF0-40EE-AB44-C05703D69E0B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="67">
   <si>
     <t>R</t>
   </si>
@@ -211,6 +211,30 @@
   </si>
   <si>
     <t>PD30PD20PD20PD20PD20H</t>
+  </si>
+  <si>
+    <t>$AMJ000500330001</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>GD50GD60LR50CR60BT11CR61BT19CR62BT27CR63</t>
+  </si>
+  <si>
+    <t>BT35LR61SR70LR62SR71LR63SR72PD70HLR60</t>
+  </si>
+  <si>
+    <t>SR70LR62SR71LR63SR72PD70HLR60SR70LR61</t>
+  </si>
+  <si>
+    <t>SR71LR63SR72PD70HLR60SR70LR61SR71LR62</t>
+  </si>
+  <si>
+    <t>SR72PD70H</t>
   </si>
 </sst>
 </file>
@@ -673,7 +697,7 @@
         <v>11</v>
       </c>
       <c r="O2" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P2" s="6">
         <v>0</v>
@@ -684,13 +708,13 @@
         <v>1</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="O3" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P3" s="6">
         <v>0</v>
@@ -711,16 +735,16 @@
         <v>2</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O4" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P4" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -731,16 +755,16 @@
         <v>3</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O5" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P5" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -756,16 +780,16 @@
         <v>4</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="O6" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P6" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -776,16 +800,16 @@
         <v>5</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O7" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P7" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -800,16 +824,16 @@
         <v>6</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="O8" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P8" s="6">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -817,16 +841,16 @@
         <v>7</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>0</v>
       </c>
       <c r="O9" s="6">
+        <v>6</v>
+      </c>
+      <c r="P9" s="6">
         <v>2</v>
-      </c>
-      <c r="P9" s="6">
-        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -838,16 +862,16 @@
         <v>8</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="O10" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
@@ -858,16 +882,16 @@
         <v>9</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O11" s="6">
+        <v>6</v>
+      </c>
+      <c r="P11" s="6">
         <v>3</v>
-      </c>
-      <c r="P11" s="6">
-        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
@@ -875,11 +899,17 @@
         <v>10</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
+        <v>61</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="O12" s="5">
+        <v>3</v>
+      </c>
+      <c r="P12" s="5">
+        <v>5</v>
+      </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -888,10 +918,18 @@
       <c r="L13">
         <v>11</v>
       </c>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
+      <c r="M13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O13" s="5">
+        <v>6</v>
+      </c>
+      <c r="P13" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -900,10 +938,18 @@
       <c r="L14">
         <v>12</v>
       </c>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
+      <c r="M14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O14" s="5">
+        <v>7</v>
+      </c>
+      <c r="P14" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -912,10 +958,18 @@
       <c r="L15">
         <v>13</v>
       </c>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
+      <c r="M15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O15" s="5">
+        <v>6</v>
+      </c>
+      <c r="P15" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -924,10 +978,18 @@
       <c r="L16">
         <v>14</v>
       </c>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
+      <c r="M16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O16" s="5">
+        <v>7</v>
+      </c>
+      <c r="P16" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -936,10 +998,18 @@
       <c r="L17">
         <v>15</v>
       </c>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
+      <c r="M17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O17" s="5">
+        <v>6</v>
+      </c>
+      <c r="P17" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -948,10 +1018,18 @@
       <c r="L18">
         <v>16</v>
       </c>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
+      <c r="M18" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O18" s="5">
+        <v>7</v>
+      </c>
+      <c r="P18" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -960,10 +1038,18 @@
       <c r="L19">
         <v>17</v>
       </c>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
+      <c r="M19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O19" s="5">
+        <v>7</v>
+      </c>
+      <c r="P19" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -972,7 +1058,9 @@
       <c r="L20">
         <v>18</v>
       </c>
-      <c r="M20" s="5"/>
+      <c r="M20" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
       <c r="P20" s="5"/>
@@ -984,28 +1072,52 @@
       <c r="L21">
         <v>19</v>
       </c>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
+      <c r="M21" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="O21" s="5">
+        <v>6</v>
+      </c>
+      <c r="P21" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L22">
         <v>20</v>
       </c>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="6"/>
+      <c r="M22" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N22" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O22" s="6">
+        <v>7</v>
+      </c>
+      <c r="P22" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L23">
         <v>21</v>
       </c>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="6"/>
-      <c r="P23" s="6"/>
+      <c r="M23" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O23" s="6">
+        <v>6</v>
+      </c>
+      <c r="P23" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1014,19 +1126,35 @@
       <c r="L24">
         <v>22</v>
       </c>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
+      <c r="M24" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N24" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6">
+        <v>7</v>
+      </c>
+      <c r="P24" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L25">
         <v>23</v>
       </c>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
+      <c r="M25" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O25" s="6">
+        <v>6</v>
+      </c>
+      <c r="P25" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1035,10 +1163,18 @@
       <c r="L26">
         <v>24</v>
       </c>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
+      <c r="M26" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N26" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6">
+        <v>7</v>
+      </c>
+      <c r="P26" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
@@ -1047,10 +1183,18 @@
       <c r="L27">
         <v>25</v>
       </c>
-      <c r="M27" s="6"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="6"/>
-      <c r="P27" s="6"/>
+      <c r="M27" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="O27" s="6">
+        <v>7</v>
+      </c>
+      <c r="P27" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
@@ -1059,7 +1203,9 @@
       <c r="L28">
         <v>26</v>
       </c>
-      <c r="M28" s="6"/>
+      <c r="M28" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
@@ -1071,10 +1217,18 @@
       <c r="L29">
         <v>27</v>
       </c>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
+      <c r="M29" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N29" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O29" s="6">
+        <v>6</v>
+      </c>
+      <c r="P29" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
@@ -1083,10 +1237,18 @@
       <c r="L30">
         <v>28</v>
       </c>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
+      <c r="M30" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N30" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O30" s="6">
+        <v>7</v>
+      </c>
+      <c r="P30" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
@@ -1095,28 +1257,52 @@
       <c r="L31">
         <v>29</v>
       </c>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
+      <c r="M31" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O31" s="6">
+        <v>6</v>
+      </c>
+      <c r="P31" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L32">
         <v>30</v>
       </c>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
+      <c r="M32" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O32" s="5">
+        <v>7</v>
+      </c>
+      <c r="P32" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L33">
         <v>31</v>
       </c>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
+      <c r="M33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O33" s="5">
+        <v>6</v>
+      </c>
+      <c r="P33" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
@@ -1125,19 +1311,35 @@
       <c r="L34">
         <v>32</v>
       </c>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
+      <c r="M34" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N34" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O34" s="5">
+        <v>7</v>
+      </c>
+      <c r="P34" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L35">
         <v>33</v>
       </c>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
+      <c r="M35" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O35" s="5">
+        <v>7</v>
+      </c>
+      <c r="P35" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
@@ -1146,7 +1348,9 @@
       <c r="L36">
         <v>34</v>
       </c>
-      <c r="M36" s="5"/>
+      <c r="M36" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="N36" s="5"/>
       <c r="O36" s="5"/>
       <c r="P36" s="5"/>
@@ -1158,10 +1362,18 @@
       <c r="L37">
         <v>35</v>
       </c>
-      <c r="M37" s="5"/>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
+      <c r="M37" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N37" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O37" s="5">
+        <v>6</v>
+      </c>
+      <c r="P37" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
@@ -1170,10 +1382,18 @@
       <c r="L38">
         <v>36</v>
       </c>
-      <c r="M38" s="5"/>
-      <c r="N38" s="5"/>
-      <c r="O38" s="5"/>
-      <c r="P38" s="5"/>
+      <c r="M38" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N38" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O38" s="5">
+        <v>7</v>
+      </c>
+      <c r="P38" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
@@ -1182,10 +1402,18 @@
       <c r="L39">
         <v>37</v>
       </c>
-      <c r="M39" s="5"/>
-      <c r="N39" s="5"/>
-      <c r="O39" s="5"/>
-      <c r="P39" s="5"/>
+      <c r="M39" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N39" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O39" s="5">
+        <v>6</v>
+      </c>
+      <c r="P39" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
@@ -1194,10 +1422,18 @@
       <c r="L40">
         <v>38</v>
       </c>
-      <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
-      <c r="O40" s="5"/>
-      <c r="P40" s="5"/>
+      <c r="M40" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N40" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O40" s="5">
+        <v>7</v>
+      </c>
+      <c r="P40" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
@@ -1206,10 +1442,18 @@
       <c r="L41">
         <v>39</v>
       </c>
-      <c r="M41" s="5"/>
-      <c r="N41" s="5"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
+      <c r="M41" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N41" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O41" s="5">
+        <v>6</v>
+      </c>
+      <c r="P41" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
@@ -1218,10 +1462,18 @@
       <c r="L42">
         <v>40</v>
       </c>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="6"/>
+      <c r="M42" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N42" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="O42" s="6">
+        <v>7</v>
+      </c>
+      <c r="P42" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
@@ -1230,10 +1482,18 @@
       <c r="L43">
         <v>41</v>
       </c>
-      <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
-      <c r="O43" s="6"/>
-      <c r="P43" s="6"/>
+      <c r="M43" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="O43" s="6">
+        <v>7</v>
+      </c>
+      <c r="P43" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
@@ -1242,7 +1502,9 @@
       <c r="L44">
         <v>42</v>
       </c>
-      <c r="M44" s="6"/>
+      <c r="M44" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
       <c r="P44" s="6"/>
@@ -1290,6 +1552,9 @@
       <c r="A49" t="s">
         <v>45</v>
       </c>
+      <c r="G49" t="s">
+        <v>59</v>
+      </c>
       <c r="L49">
         <v>47</v>
       </c>
@@ -1302,6 +1567,9 @@
       <c r="A50" t="s">
         <v>42</v>
       </c>
+      <c r="G50" t="s">
+        <v>62</v>
+      </c>
       <c r="L50">
         <v>48</v>
       </c>
@@ -1314,6 +1582,9 @@
       <c r="A51" t="s">
         <v>43</v>
       </c>
+      <c r="G51" t="s">
+        <v>63</v>
+      </c>
       <c r="L51">
         <v>49</v>
       </c>
@@ -1326,6 +1597,9 @@
       <c r="A52" t="s">
         <v>44</v>
       </c>
+      <c r="G52" t="s">
+        <v>64</v>
+      </c>
       <c r="L52">
         <v>50</v>
       </c>
@@ -1338,6 +1612,9 @@
       <c r="A53" t="s">
         <v>7</v>
       </c>
+      <c r="G53" t="s">
+        <v>65</v>
+      </c>
       <c r="L53">
         <v>51</v>
       </c>
@@ -1350,6 +1627,9 @@
       <c r="A54" t="s">
         <v>27</v>
       </c>
+      <c r="G54" t="s">
+        <v>66</v>
+      </c>
       <c r="L54">
         <v>52</v>
       </c>
@@ -1362,6 +1642,9 @@
       <c r="A55" t="s">
         <v>28</v>
       </c>
+      <c r="G55" t="s">
+        <v>7</v>
+      </c>
       <c r="L55">
         <v>53</v>
       </c>
@@ -1374,6 +1657,9 @@
       <c r="A56" t="s">
         <v>47</v>
       </c>
+      <c r="G56" t="s">
+        <v>27</v>
+      </c>
       <c r="L56">
         <v>54</v>
       </c>
@@ -1383,6 +1669,9 @@
       <c r="P56" s="5"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G57" t="s">
+        <v>28</v>
+      </c>
       <c r="L57">
         <v>55</v>
       </c>
@@ -1392,6 +1681,9 @@
       <c r="P57" s="5"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G58" t="s">
+        <v>47</v>
+      </c>
       <c r="L58">
         <v>56</v>
       </c>

</xml_diff>